<commit_message>
made nomi the priority
</commit_message>
<xml_diff>
--- a/drive-time-locator/Backend/locations_with_coords.xlsx
+++ b/drive-time-locator/Backend/locations_with_coords.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olivier.d\.vscode\closest-dealer-api\drive-time-locator\Backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3909926A-C25C-43AB-8F97-C0FE0D46F3BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6E3A6C3-37B2-4ACF-A466-35A2DC3777A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1520" yWindow="1520" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="140">
   <si>
     <t>Name</t>
   </si>
@@ -245,12 +245,6 @@
   </si>
   <si>
     <t>SUN SERVICE SPECIALISTS LLC</t>
-  </si>
-  <si>
-    <t>8885857861</t>
-  </si>
-  <si>
-    <t>801 PRESSLEY RD STE 100-C, CHARLOTTE, NC, 28217</t>
   </si>
   <si>
     <t>CLEAN ENERGY INNOVATORS LLC</t>
@@ -857,8 +851,8 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:E1000"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:E999"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="12.25" customWidth="1"/>
@@ -1277,395 +1271,379 @@
     </row>
     <row r="25" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D25" s="2">
-        <v>35.188482999999998</v>
+        <v>47.371457999999997</v>
       </c>
       <c r="E25" s="2">
-        <v>-80.893687</v>
+        <v>-122.168651</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D26" s="2">
-        <v>47.371457999999997</v>
+        <v>37.9407</v>
       </c>
       <c r="E26" s="2">
-        <v>-122.168651</v>
+        <v>-78.636679999999998</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D27" s="2">
-        <v>37.9407</v>
+        <v>41.323565000000002</v>
       </c>
       <c r="E27" s="2">
-        <v>-78.636679999999998</v>
+        <v>-82.490208999999993</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D28" s="2">
-        <v>41.323565000000002</v>
+        <v>29.694703000000001</v>
       </c>
       <c r="E28" s="2">
-        <v>-82.490208999999993</v>
+        <v>-98.116089000000002</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D29" s="2">
-        <v>29.694703000000001</v>
+        <v>39.219279999999998</v>
       </c>
       <c r="E29" s="2">
-        <v>-98.116089000000002</v>
+        <v>-86.620096000000004</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D30" s="2">
-        <v>39.219279999999998</v>
+        <v>39.89385</v>
       </c>
       <c r="E30" s="2">
-        <v>-86.620096000000004</v>
+        <v>-86.246138000000002</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D31" s="2">
-        <v>39.89385</v>
+        <v>35.973011</v>
       </c>
       <c r="E31" s="2">
-        <v>-86.246138000000002</v>
+        <v>-83.969471999999996</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D32" s="2">
-        <v>35.973011</v>
+        <v>38.898076000000003</v>
       </c>
       <c r="E32" s="2">
-        <v>-83.969471999999996</v>
+        <v>-121.071247</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D33" s="2">
-        <v>38.898076000000003</v>
+        <v>40.966545000000004</v>
       </c>
       <c r="E33" s="2">
-        <v>-121.071247</v>
+        <v>-81.788776999999996</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D34" s="2">
-        <v>40.966545000000004</v>
+        <v>33.012175999999997</v>
       </c>
       <c r="E34" s="2">
-        <v>-81.788776999999996</v>
+        <v>-80.182766000000001</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D35" s="2">
-        <v>33.012175999999997</v>
+        <v>39.306282000000003</v>
       </c>
       <c r="E35" s="2">
-        <v>-80.182766000000001</v>
+        <v>-84.381606000000005</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D36" s="2">
-        <v>39.306282000000003</v>
+        <v>35.895916</v>
       </c>
       <c r="E36" s="2">
-        <v>-84.381606000000005</v>
+        <v>-78.745880999999997</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D37" s="2">
-        <v>35.895916</v>
+        <v>38.036141000000001</v>
       </c>
       <c r="E37" s="2">
-        <v>-78.745880999999997</v>
+        <v>-78.482369000000006</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D38" s="2">
-        <v>38.036141000000001</v>
+        <v>41.644714</v>
       </c>
       <c r="E38" s="2">
-        <v>-78.482369000000006</v>
+        <v>-88.616303000000002</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D39" s="2">
-        <v>41.644714</v>
+        <v>37.311083000000004</v>
       </c>
       <c r="E39" s="2">
-        <v>-88.616303000000002</v>
+        <v>-107.858233</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D40" s="2">
-        <v>37.311083000000004</v>
+        <v>39.789189999999998</v>
       </c>
       <c r="E40" s="2">
-        <v>-107.858233</v>
+        <v>-104.950523</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D41" s="2">
-        <v>39.789189999999998</v>
+        <v>40.584440999999998</v>
       </c>
       <c r="E41" s="2">
-        <v>-104.950523</v>
+        <v>-105.078982</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D42" s="2">
-        <v>40.584440999999998</v>
+        <v>36.226163999999997</v>
       </c>
       <c r="E42" s="2">
-        <v>-105.078982</v>
+        <v>-86.629830999999996</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D43" s="2">
-        <v>36.226163999999997</v>
+        <v>39.748579999999997</v>
       </c>
       <c r="E43" s="2">
-        <v>-86.629830999999996</v>
+        <v>-105.07538</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D44" s="2">
-        <v>39.748579999999997</v>
+        <v>28.81718</v>
       </c>
       <c r="E44" s="2">
-        <v>-105.07538</v>
+        <v>-81.848889999999997</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="B45" s="2" t="s">
+      <c r="A45" t="s">
+        <v>74</v>
+      </c>
+      <c r="B45" t="s">
         <v>135</v>
       </c>
-      <c r="C45" s="2" t="s">
+      <c r="C45" t="s">
         <v>136</v>
       </c>
-      <c r="D45" s="2">
-        <v>28.81718</v>
-      </c>
-      <c r="E45" s="2">
-        <v>-81.848889999999997</v>
+      <c r="D45">
+        <v>35.174399899999997</v>
+      </c>
+      <c r="E45">
+        <v>-80.904181699999995</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>74</v>
+        <v>138</v>
       </c>
       <c r="B46" t="s">
         <v>137</v>
       </c>
       <c r="C46" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D46">
-        <v>35.174399899999997</v>
+        <v>42.96716</v>
       </c>
       <c r="E46">
-        <v>-80.904181699999995</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
-        <v>140</v>
-      </c>
-      <c r="B47" t="s">
-        <v>139</v>
-      </c>
-      <c r="C47" t="s">
-        <v>141</v>
-      </c>
-      <c r="D47">
-        <v>42.96716</v>
-      </c>
-      <c r="E47">
         <v>-85.962729999999993</v>
       </c>
     </row>
+    <row r="47" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="48" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="49" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="50" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -2618,11 +2596,10 @@
     <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:E45 A48:E1000" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:E24 A47:E999 A25:E44" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Better multi threading and logs
</commit_message>
<xml_diff>
--- a/drive-time-locator/Backend/locations_with_coords.xlsx
+++ b/drive-time-locator/Backend/locations_with_coords.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olivier.d\.vscode\closest-dealer-api\drive-time-locator\Backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6E3A6C3-37B2-4ACF-A466-35A2DC3777A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDEB179D-B354-4BB6-A57E-0DA105F57361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1520" yWindow="1520" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="149">
   <si>
     <t>Name</t>
   </si>
@@ -440,12 +440,42 @@
   </si>
   <si>
     <t>7208 Timbercreek Drive Allendale, MI 49401</t>
+  </si>
+  <si>
+    <t>Solar Wiz LLC</t>
+  </si>
+  <si>
+    <t>(602) 556-8406</t>
+  </si>
+  <si>
+    <t>1755 N PEBBLE CREEK PKWY GOODYEAR, AZ 85395-2532 US</t>
+  </si>
+  <si>
+    <t>ELAN ELECTRIC INC.</t>
+  </si>
+  <si>
+    <t>(928) 925-7937</t>
+  </si>
+  <si>
+    <t>7760 E STATE ROUTE 69, PRESCOTT VALLEY, AZ, 86314</t>
+  </si>
+  <si>
+    <t>Sun Power Energy</t>
+  </si>
+  <si>
+    <t>(719) 238-4554</t>
+  </si>
+  <si>
+    <t>2090 COPLEY RD, COLORADO SPRINGS, CO, 80920</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="168" formatCode="0.00000"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -503,12 +533,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
@@ -524,6 +555,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1643,24 +1678,72 @@
         <v>-85.962729999999993</v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="48" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="49" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="50" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="51" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="52" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="53" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="54" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="55" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="56" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="57" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="58" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="59" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="60" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="61" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="62" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="63" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="64" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="47" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>140</v>
+      </c>
+      <c r="B47" t="s">
+        <v>141</v>
+      </c>
+      <c r="C47" t="s">
+        <v>142</v>
+      </c>
+      <c r="D47">
+        <v>33.466299999999997</v>
+      </c>
+      <c r="E47">
+        <v>-112.38775</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>143</v>
+      </c>
+      <c r="B48" t="s">
+        <v>144</v>
+      </c>
+      <c r="C48" t="s">
+        <v>145</v>
+      </c>
+      <c r="D48" s="3">
+        <v>34.587166000000003</v>
+      </c>
+      <c r="E48" s="3">
+        <v>-112.329256</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>146</v>
+      </c>
+      <c r="B49" t="s">
+        <v>147</v>
+      </c>
+      <c r="C49" t="s">
+        <v>148</v>
+      </c>
+      <c r="D49" s="3">
+        <v>38.957118000000001</v>
+      </c>
+      <c r="E49" s="3">
+        <v>-104.789243</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="51" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="52" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="53" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="54" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="55" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="56" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="57" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="58" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="59" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="60" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="61" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="62" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="63" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="64" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="65" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="66" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="67" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -2599,7 +2682,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:E24 A47:E999 A25:E44" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:E24 A50:E999 A25:E44" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Removed Augustine Solar LLC
</commit_message>
<xml_diff>
--- a/drive-time-locator/Backend/locations_with_coords.xlsx
+++ b/drive-time-locator/Backend/locations_with_coords.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olivier.d\.vscode\closest-dealer-api\drive-time-locator\Backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B97A7B66-909A-4BF9-BBEF-8E61A9AE3201}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19004F0B-E85A-4F42-B903-2983E33272CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="148">
   <si>
     <t>Name</t>
   </si>
@@ -410,15 +410,6 @@
   </si>
   <si>
     <t>801 PRESSLEY RD STE 100-C CHARLOTTE, NC 28217 US</t>
-  </si>
-  <si>
-    <t>(616) 219-0457</t>
-  </si>
-  <si>
-    <t>Augustine Solar LLC</t>
-  </si>
-  <si>
-    <t>7208 Timbercreek Drive Allendale, MI 49401</t>
   </si>
   <si>
     <t>Solar Wiz LLC</t>
@@ -557,7 +548,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -575,10 +566,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -906,7 +893,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:F998"/>
+  <dimension ref="A1:F997"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -933,7 +920,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -941,7 +928,7 @@
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>6</v>
@@ -953,7 +940,7 @@
         <v>-95.559602999999996</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1604,7 +1591,7 @@
     </row>
     <row r="41" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>122</v>
@@ -1619,12 +1606,12 @@
         <v>-86.629830999999996</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>124</v>
@@ -1639,12 +1626,12 @@
         <v>-105.07538</v>
       </c>
       <c r="F42" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>126</v>
@@ -1659,7 +1646,7 @@
         <v>-81.848889999999997</v>
       </c>
       <c r="F43" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -1679,24 +1666,24 @@
         <v>-80.904181699999995</v>
       </c>
       <c r="F44" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
+        <v>130</v>
+      </c>
+      <c r="B45" t="s">
         <v>131</v>
-      </c>
-      <c r="B45" t="s">
-        <v>130</v>
       </c>
       <c r="C45" t="s">
         <v>132</v>
       </c>
       <c r="D45">
-        <v>42.96716</v>
+        <v>33.466299999999997</v>
       </c>
       <c r="E45">
-        <v>-85.962729999999993</v>
+        <v>-112.38775</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -1709,11 +1696,11 @@
       <c r="C46" t="s">
         <v>135</v>
       </c>
-      <c r="D46">
-        <v>33.466299999999997</v>
-      </c>
-      <c r="E46">
-        <v>-112.38775</v>
+      <c r="D46" s="3">
+        <v>34.587166000000003</v>
+      </c>
+      <c r="E46" s="3">
+        <v>-112.329256</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -1727,29 +1714,13 @@
         <v>138</v>
       </c>
       <c r="D47" s="3">
-        <v>34.587166000000003</v>
+        <v>38.957118000000001</v>
       </c>
       <c r="E47" s="3">
-        <v>-112.329256</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
-        <v>139</v>
-      </c>
-      <c r="B48" t="s">
-        <v>140</v>
-      </c>
-      <c r="C48" t="s">
-        <v>141</v>
-      </c>
-      <c r="D48" s="3">
-        <v>38.957118000000001</v>
-      </c>
-      <c r="E48" s="3">
         <v>-104.789243</v>
       </c>
     </row>
+    <row r="48" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="49" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="50" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="51" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -2699,11 +2670,10 @@
     <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:E1 A49:E998 A24:E40 A3:E23 A2 C2:E2 B43 D43:E43 B42:E42 B41:E41" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:E1 A48:E997 A24:E40 A3:E23 A2 C2:E2 B43 D43:E43 B42:E42 B41:E41" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added a new dealer
</commit_message>
<xml_diff>
--- a/drive-time-locator/Backend/locations_with_coords.xlsx
+++ b/drive-time-locator/Backend/locations_with_coords.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olivier.d\.vscode\closest-dealer-api\drive-time-locator\Backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19004F0B-E85A-4F42-B903-2983E33272CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AA53981-E26A-442F-B987-1B22FB0FEA76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="152">
   <si>
     <t>Name</t>
   </si>
@@ -464,6 +464,18 @@
   </si>
   <si>
     <t>KW ENERGY SOLUTIONS, LLC</t>
+  </si>
+  <si>
+    <t>537 PARKDALE DR SALEM, VA 24153 US</t>
+  </si>
+  <si>
+    <t>TREVOR WOODSON DBA JILA SALES</t>
+  </si>
+  <si>
+    <t>(540) 200-7797</t>
+  </si>
+  <si>
+    <t>Willing to travel 300 miles from Salem </t>
   </si>
 </sst>
 </file>
@@ -1720,7 +1732,26 @@
         <v>-104.789243</v>
       </c>
     </row>
-    <row r="48" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="48" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>149</v>
+      </c>
+      <c r="B48" t="s">
+        <v>150</v>
+      </c>
+      <c r="C48" t="s">
+        <v>148</v>
+      </c>
+      <c r="D48">
+        <v>37.304490000000001</v>
+      </c>
+      <c r="E48">
+        <v>-80.036469999999994</v>
+      </c>
+      <c r="F48" t="s">
+        <v>151</v>
+      </c>
+    </row>
     <row r="49" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="50" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="51" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -2672,8 +2703,9 @@
     <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:E1 A48:E997 A24:E40 A3:E23 A2 C2:E2 B43 D43:E43 B42:E42 B41:E41" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:E1 A49:E997 A24:E40 A3:E23 A2 C2:E2 B43 D43:E43 B42:E42 B41:E41" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Changed YOUR HOME SOLAR LLC's number to their new one
</commit_message>
<xml_diff>
--- a/drive-time-locator/Backend/locations_with_coords.xlsx
+++ b/drive-time-locator/Backend/locations_with_coords.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olivier.d\.vscode\closest-dealer-api\drive-time-locator\Backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AA53981-E26A-442F-B987-1B22FB0FEA76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{606CB58F-49F4-4EBD-83B1-F9CD1169EE47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-1428" yWindow="-11580" windowWidth="14400" windowHeight="8172" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -226,9 +226,6 @@
     <t>YOUR HOME SOLAR LLC</t>
   </si>
   <si>
-    <t>865-236-3193</t>
-  </si>
-  <si>
     <t>6210 CARDWELL RD, CORRYTON, TN, 37721-3715</t>
   </si>
   <si>
@@ -476,6 +473,9 @@
   </si>
   <si>
     <t>Willing to travel 300 miles from Salem </t>
+  </si>
+  <si>
+    <t>865-314-7040</t>
   </si>
 </sst>
 </file>
@@ -932,7 +932,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -940,7 +940,7 @@
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>6</v>
@@ -952,7 +952,7 @@
         <v>-95.559602999999996</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1300,10 +1300,10 @@
         <v>67</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>69</v>
       </c>
       <c r="D23" s="2">
         <v>36.153689999999997</v>
@@ -1314,13 +1314,13 @@
     </row>
     <row r="24" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="C24" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>73</v>
       </c>
       <c r="D24" s="2">
         <v>47.371457999999997</v>
@@ -1331,13 +1331,13 @@
     </row>
     <row r="25" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="C25" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>76</v>
       </c>
       <c r="D25" s="2">
         <v>37.9407</v>
@@ -1348,13 +1348,13 @@
     </row>
     <row r="26" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="C26" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>79</v>
       </c>
       <c r="D26" s="2">
         <v>41.323565000000002</v>
@@ -1365,13 +1365,13 @@
     </row>
     <row r="27" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="C27" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>82</v>
       </c>
       <c r="D27" s="2">
         <v>29.694703000000001</v>
@@ -1382,13 +1382,13 @@
     </row>
     <row r="28" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="C28" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>85</v>
       </c>
       <c r="D28" s="2">
         <v>39.219279999999998</v>
@@ -1399,13 +1399,13 @@
     </row>
     <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="C29" s="2" t="s">
         <v>87</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>88</v>
       </c>
       <c r="D29" s="2">
         <v>39.89385</v>
@@ -1416,13 +1416,13 @@
     </row>
     <row r="30" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="C30" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>91</v>
       </c>
       <c r="D30" s="2">
         <v>35.973011</v>
@@ -1433,13 +1433,13 @@
     </row>
     <row r="31" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B31" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="C31" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>94</v>
       </c>
       <c r="D31" s="2">
         <v>38.898076000000003</v>
@@ -1450,13 +1450,13 @@
     </row>
     <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="C32" s="2" t="s">
         <v>96</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>97</v>
       </c>
       <c r="D32" s="2">
         <v>40.966545000000004</v>
@@ -1467,13 +1467,13 @@
     </row>
     <row r="33" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="C33" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>100</v>
       </c>
       <c r="D33" s="2">
         <v>33.012175999999997</v>
@@ -1484,13 +1484,13 @@
     </row>
     <row r="34" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="C34" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="D34" s="2">
         <v>39.306282000000003</v>
@@ -1501,13 +1501,13 @@
     </row>
     <row r="35" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="C35" s="2" t="s">
         <v>105</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>106</v>
       </c>
       <c r="D35" s="2">
         <v>35.895916</v>
@@ -1518,13 +1518,13 @@
     </row>
     <row r="36" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="C36" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>109</v>
       </c>
       <c r="D36" s="2">
         <v>38.036141000000001</v>
@@ -1535,13 +1535,13 @@
     </row>
     <row r="37" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="C37" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>112</v>
       </c>
       <c r="D37" s="2">
         <v>41.644714</v>
@@ -1552,13 +1552,13 @@
     </row>
     <row r="38" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="C38" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>115</v>
       </c>
       <c r="D38" s="2">
         <v>37.311083000000004</v>
@@ -1569,13 +1569,13 @@
     </row>
     <row r="39" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="C39" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>118</v>
       </c>
       <c r="D39" s="2">
         <v>39.789189999999998</v>
@@ -1586,13 +1586,13 @@
     </row>
     <row r="40" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="C40" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>121</v>
       </c>
       <c r="D40" s="2">
         <v>40.584440999999998</v>
@@ -1603,13 +1603,13 @@
     </row>
     <row r="41" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B41" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="D41" s="2">
         <v>36.226163999999997</v>
@@ -1618,18 +1618,18 @@
         <v>-86.629830999999996</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B42" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>124</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>125</v>
       </c>
       <c r="D42" s="2">
         <v>39.748579999999997</v>
@@ -1638,18 +1638,18 @@
         <v>-105.07538</v>
       </c>
       <c r="F42" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B43" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>126</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>127</v>
       </c>
       <c r="D43" s="2">
         <v>28.81718</v>
@@ -1658,18 +1658,18 @@
         <v>-81.848889999999997</v>
       </c>
       <c r="F43" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B44" t="s">
+        <v>127</v>
+      </c>
+      <c r="C44" t="s">
         <v>128</v>
-      </c>
-      <c r="C44" t="s">
-        <v>129</v>
       </c>
       <c r="D44">
         <v>35.174399899999997</v>
@@ -1678,18 +1678,18 @@
         <v>-80.904181699999995</v>
       </c>
       <c r="F44" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
+        <v>129</v>
+      </c>
+      <c r="B45" t="s">
         <v>130</v>
       </c>
-      <c r="B45" t="s">
+      <c r="C45" t="s">
         <v>131</v>
-      </c>
-      <c r="C45" t="s">
-        <v>132</v>
       </c>
       <c r="D45">
         <v>33.466299999999997</v>
@@ -1700,13 +1700,13 @@
     </row>
     <row r="46" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
+        <v>132</v>
+      </c>
+      <c r="B46" t="s">
         <v>133</v>
       </c>
-      <c r="B46" t="s">
+      <c r="C46" t="s">
         <v>134</v>
-      </c>
-      <c r="C46" t="s">
-        <v>135</v>
       </c>
       <c r="D46" s="3">
         <v>34.587166000000003</v>
@@ -1717,13 +1717,13 @@
     </row>
     <row r="47" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
+        <v>135</v>
+      </c>
+      <c r="B47" t="s">
         <v>136</v>
       </c>
-      <c r="B47" t="s">
+      <c r="C47" t="s">
         <v>137</v>
-      </c>
-      <c r="C47" t="s">
-        <v>138</v>
       </c>
       <c r="D47" s="3">
         <v>38.957118000000001</v>
@@ -1734,13 +1734,13 @@
     </row>
     <row r="48" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
+        <v>148</v>
+      </c>
+      <c r="B48" t="s">
         <v>149</v>
       </c>
-      <c r="B48" t="s">
-        <v>150</v>
-      </c>
       <c r="C48" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D48">
         <v>37.304490000000001</v>
@@ -1749,7 +1749,7 @@
         <v>-80.036469999999994</v>
       </c>
       <c r="F48" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -2705,7 +2705,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:E1 A49:E997 A24:E40 A3:E23 A2 C2:E2 B43 D43:E43 B42:E42 B41:E41" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:E1 A49:E997 A24:E40 A3:E22 A2 C2:E2 B43 D43:E43 B42:E42 B41:E41 C23:E23" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Changed some address that were defaulted to billing instead of shipping which should be a more accurate gauge of working distance.
</commit_message>
<xml_diff>
--- a/drive-time-locator/Backend/locations_with_coords.xlsx
+++ b/drive-time-locator/Backend/locations_with_coords.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olivier.d\.vscode\closest-dealer-api\drive-time-locator\Backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{606CB58F-49F4-4EBD-83B1-F9CD1169EE47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{482BFCD0-F7E9-44C9-AD8A-EC436AE14816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-1428" yWindow="-11580" windowWidth="14400" windowHeight="8172" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -121,9 +134,6 @@
     <t>4073777437</t>
   </si>
   <si>
-    <t>932 KENMORE AVE, BUFFALO, NY, 14216-1462</t>
-  </si>
-  <si>
     <t>All Circuit Electrical L.L.C.</t>
   </si>
   <si>
@@ -139,9 +149,6 @@
     <t>8083068919</t>
   </si>
   <si>
-    <t>7511 KEKAA ST, HONOLULU, HI, 96825-2805</t>
-  </si>
-  <si>
     <t>MICHIGAN SOLAR SOLUTIONS INC</t>
   </si>
   <si>
@@ -157,9 +164,6 @@
     <t>6023696969</t>
   </si>
   <si>
-    <t>6150 W CHANDLER BLVD #17, CHANDLER, AZ, 85226</t>
-  </si>
-  <si>
     <t>Riverside Electric</t>
   </si>
   <si>
@@ -319,9 +323,6 @@
     <t>854-219-2357</t>
   </si>
   <si>
-    <t>180 GRANTON EDGE LN, SUMMERVILLE, SC, 29486</t>
-  </si>
-  <si>
     <t>PRO SOLAR SOLUTIONS LLC</t>
   </si>
   <si>
@@ -476,6 +477,18 @@
   </si>
   <si>
     <t>865-314-7040</t>
+  </si>
+  <si>
+    <t>19400 Florida 44 Eustis, FL 32736 United States</t>
+  </si>
+  <si>
+    <t>86 IHO IHO Place WAHIAWA, HI 96786</t>
+  </si>
+  <si>
+    <t>1400 E Southern Ave STE 130 Tempe, AZ 85282 United States</t>
+  </si>
+  <si>
+    <t>5207 Hawkins Meadow Ct, Charlotte, NC 28213, USA</t>
   </si>
 </sst>
 </file>
@@ -932,7 +945,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -940,7 +953,7 @@
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>6</v>
@@ -952,7 +965,7 @@
         <v>-95.559602999999996</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1099,24 +1112,24 @@
         <v>32</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>33</v>
+        <v>148</v>
       </c>
       <c r="D11" s="2">
-        <v>42.958297000000002</v>
+        <v>28.850374804966101</v>
       </c>
       <c r="E11" s="2">
-        <v>-78.852472000000006</v>
+        <v>-81.632558139953304</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>36</v>
       </c>
       <c r="D12" s="2">
         <v>35.74174</v>
@@ -1127,30 +1140,30 @@
     </row>
     <row r="13" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="C13" s="2" t="s">
-        <v>39</v>
+        <v>149</v>
       </c>
       <c r="D13" s="2">
-        <v>21.405719999999999</v>
+        <v>21.497420327698102</v>
       </c>
       <c r="E13" s="2">
-        <v>-157.78939600000001</v>
+        <v>-158.02047783221599</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>40</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>42</v>
       </c>
       <c r="D14" s="2">
         <v>42.569713</v>
@@ -1161,30 +1174,30 @@
     </row>
     <row r="15" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>45</v>
+        <v>150</v>
       </c>
       <c r="D15" s="2">
-        <v>33.310045000000002</v>
+        <v>33.393993764255498</v>
       </c>
       <c r="E15" s="2">
-        <v>-111.861363</v>
+        <v>-111.915893860729</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D16" s="2">
         <v>39.262909000000001</v>
@@ -1195,13 +1208,13 @@
     </row>
     <row r="17" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D17" s="2">
         <v>21.325071999999999</v>
@@ -1212,13 +1225,13 @@
     </row>
     <row r="18" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D18" s="2">
         <v>44.092323</v>
@@ -1229,13 +1242,13 @@
     </row>
     <row r="19" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D19" s="2">
         <v>34.221238</v>
@@ -1246,13 +1259,13 @@
     </row>
     <row r="20" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D20" s="2">
         <v>37.383606999999998</v>
@@ -1263,13 +1276,13 @@
     </row>
     <row r="21" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D21" s="2">
         <v>42.467131999999999</v>
@@ -1280,13 +1293,13 @@
     </row>
     <row r="22" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D22" s="2">
         <v>41.884461999999999</v>
@@ -1297,13 +1310,13 @@
     </row>
     <row r="23" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D23" s="2">
         <v>36.153689999999997</v>
@@ -1314,13 +1327,13 @@
     </row>
     <row r="24" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D24" s="2">
         <v>47.371457999999997</v>
@@ -1331,13 +1344,13 @@
     </row>
     <row r="25" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D25" s="2">
         <v>37.9407</v>
@@ -1348,13 +1361,13 @@
     </row>
     <row r="26" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D26" s="2">
         <v>41.323565000000002</v>
@@ -1365,13 +1378,13 @@
     </row>
     <row r="27" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D27" s="2">
         <v>29.694703000000001</v>
@@ -1382,13 +1395,13 @@
     </row>
     <row r="28" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D28" s="2">
         <v>39.219279999999998</v>
@@ -1399,13 +1412,13 @@
     </row>
     <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D29" s="2">
         <v>39.89385</v>
@@ -1416,13 +1429,13 @@
     </row>
     <row r="30" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D30" s="2">
         <v>35.973011</v>
@@ -1433,13 +1446,13 @@
     </row>
     <row r="31" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D31" s="2">
         <v>38.898076000000003</v>
@@ -1450,13 +1463,13 @@
     </row>
     <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D32" s="2">
         <v>40.966545000000004</v>
@@ -1467,30 +1480,30 @@
     </row>
     <row r="33" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>99</v>
+        <v>151</v>
       </c>
       <c r="D33" s="2">
-        <v>33.012175999999997</v>
+        <v>35.294231952066198</v>
       </c>
       <c r="E33" s="2">
-        <v>-80.182766000000001</v>
+        <v>-80.678074713099704</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D34" s="2">
         <v>39.306282000000003</v>
@@ -1501,13 +1514,13 @@
     </row>
     <row r="35" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D35" s="2">
         <v>35.895916</v>
@@ -1518,13 +1531,13 @@
     </row>
     <row r="36" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D36" s="2">
         <v>38.036141000000001</v>
@@ -1535,13 +1548,13 @@
     </row>
     <row r="37" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D37" s="2">
         <v>41.644714</v>
@@ -1552,13 +1565,13 @@
     </row>
     <row r="38" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D38" s="2">
         <v>37.311083000000004</v>
@@ -1569,13 +1582,13 @@
     </row>
     <row r="39" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D39" s="2">
         <v>39.789189999999998</v>
@@ -1586,13 +1599,13 @@
     </row>
     <row r="40" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D40" s="2">
         <v>40.584440999999998</v>
@@ -1603,13 +1616,13 @@
     </row>
     <row r="41" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="D41" s="2">
         <v>36.226163999999997</v>
@@ -1618,18 +1631,18 @@
         <v>-86.629830999999996</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D42" s="2">
         <v>39.748579999999997</v>
@@ -1638,18 +1651,18 @@
         <v>-105.07538</v>
       </c>
       <c r="F42" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="D43" s="2">
         <v>28.81718</v>
@@ -1658,18 +1671,18 @@
         <v>-81.848889999999997</v>
       </c>
       <c r="F43" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B44" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C44" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="D44">
         <v>35.174399899999997</v>
@@ -1678,18 +1691,18 @@
         <v>-80.904181699999995</v>
       </c>
       <c r="F44" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B45" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C45" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D45">
         <v>33.466299999999997</v>
@@ -1700,13 +1713,13 @@
     </row>
     <row r="46" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B46" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C46" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D46" s="3">
         <v>34.587166000000003</v>
@@ -1717,13 +1730,13 @@
     </row>
     <row r="47" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B47" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C47" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D47" s="3">
         <v>38.957118000000001</v>
@@ -1734,13 +1747,13 @@
     </row>
     <row r="48" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B48" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C48" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="D48">
         <v>37.304490000000001</v>
@@ -1749,7 +1762,7 @@
         <v>-80.036469999999994</v>
       </c>
       <c r="F48" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -2705,7 +2718,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:E1 A49:E997 A24:E40 A3:E22 A2 C2:E2 B43 D43:E43 B42:E42 B41:E41 C23:E23" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:E1 A49:E997 A24:E32 A3:E10 A2 C2:E2 B43 D43:E43 B42:E42 B41:E41 C23:E23 A12:E12 A11:B11 A14:E14 A13:B13 A16:E22 A15:B15 A34:E40 A33:B33" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added 2 dealers and a numbner to Otovo for houston
</commit_message>
<xml_diff>
--- a/drive-time-locator/Backend/locations_with_coords.xlsx
+++ b/drive-time-locator/Backend/locations_with_coords.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olivier.d\.vscode\closest-dealer-api\drive-time-locator\Backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{482BFCD0-F7E9-44C9-AD8A-EC436AE14816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC974247-68AE-4286-BFC2-6DCA32E32D9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="159">
   <si>
     <t>Name</t>
   </si>
@@ -440,12 +440,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>Assigned by escalation</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
     <t>Only provides service within 100 miles</t>
   </si>
   <si>
@@ -489,6 +483,33 @@
   </si>
   <si>
     <t>5207 Hawkins Meadow Ct, Charlotte, NC 28213, USA</t>
+  </si>
+  <si>
+    <t>TRUE TEXAS SOLAR LLC</t>
+  </si>
+  <si>
+    <t>(936) 286-8325</t>
+  </si>
+  <si>
+    <t>(833) 317-6937</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number is for the Huston Area otherwise escalate. </t>
+  </si>
+  <si>
+    <t>12275 FM 1097, Willis, TX 77318, USA</t>
+  </si>
+  <si>
+    <t>True Solar LLC</t>
+  </si>
+  <si>
+    <t>(319) 329-6270</t>
+  </si>
+  <si>
+    <t>170 Greenfield Dr d, Tiffin, IA 52340, USA</t>
+  </si>
+  <si>
+    <t>This dealer covers all of iowa and some of west IL </t>
   </si>
 </sst>
 </file>
@@ -498,7 +519,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -517,6 +538,12 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF03234D"/>
+      <name val="Segoe UI"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -566,7 +593,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -576,6 +603,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
@@ -953,7 +981,7 @@
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>136</v>
+        <v>152</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>6</v>
@@ -965,7 +993,7 @@
         <v>-95.559602999999996</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>135</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1112,7 +1140,7 @@
         <v>32</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D11" s="2">
         <v>28.850374804966101</v>
@@ -1146,7 +1174,7 @@
         <v>37</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D13" s="2">
         <v>21.497420327698102</v>
@@ -1180,7 +1208,7 @@
         <v>42</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D15" s="2">
         <v>33.393993764255498</v>
@@ -1313,7 +1341,7 @@
         <v>64</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>65</v>
@@ -1486,7 +1514,7 @@
         <v>95</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D33" s="2">
         <v>35.294231952066198</v>
@@ -1616,7 +1644,7 @@
     </row>
     <row r="41" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>117</v>
@@ -1631,12 +1659,12 @@
         <v>-86.629830999999996</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>119</v>
@@ -1651,12 +1679,12 @@
         <v>-105.07538</v>
       </c>
       <c r="F42" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>121</v>
@@ -1671,7 +1699,7 @@
         <v>-81.848889999999997</v>
       </c>
       <c r="F43" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -1691,7 +1719,7 @@
         <v>-80.904181699999995</v>
       </c>
       <c r="F44" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -1747,13 +1775,13 @@
     </row>
     <row r="48" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B48" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C48" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D48">
         <v>37.304490000000001</v>
@@ -1762,25 +1790,60 @@
         <v>-80.036469999999994</v>
       </c>
       <c r="F48" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="49" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="50" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="51" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="52" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="53" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="54" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="55" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="56" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="57" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="58" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="59" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="60" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="61" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="62" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="63" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="64" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+        <v>144</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>150</v>
+      </c>
+      <c r="B49" t="s">
+        <v>151</v>
+      </c>
+      <c r="C49" t="s">
+        <v>154</v>
+      </c>
+      <c r="D49">
+        <v>30.425978374733798</v>
+      </c>
+      <c r="E49">
+        <v>-95.540459119362296</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A50" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="B50" t="s">
+        <v>156</v>
+      </c>
+      <c r="C50" t="s">
+        <v>157</v>
+      </c>
+      <c r="D50">
+        <v>41.689357431787499</v>
+      </c>
+      <c r="E50">
+        <v>-91.664268445845593</v>
+      </c>
+      <c r="F50" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="52" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="53" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="54" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="55" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="56" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="57" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="58" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="59" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="60" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="61" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="62" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="63" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="64" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="65" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="66" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="67" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -2718,7 +2781,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:E1 A49:E997 A24:E32 A3:E10 A2 C2:E2 B43 D43:E43 B42:E42 B41:E41 C23:E23 A12:E12 A11:B11 A14:E14 A13:B13 A16:E22 A15:B15 A34:E40 A33:B33" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:E1 A51:E997 A24:E32 A3:E10 A2 C2:E2 B43 D43:E43 B42:E42 B41:E41 C23:E23 A12:E12 A11:B11 A14:E14 A13:B13 A16:E22 A15:B15 A34:E40 A33:B33" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Changed Drake Solars Number and added a new note to Otovo mentioning it covers all of Cali
</commit_message>
<xml_diff>
--- a/drive-time-locator/Backend/locations_with_coords.xlsx
+++ b/drive-time-locator/Backend/locations_with_coords.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olivier.d\.vscode\closest-dealer-api\drive-time-locator\Backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FDE5B23-F3C4-46F6-B2E4-FA61209A7232}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0519946-D867-4DF7-8B21-0C0802DFEE28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="159">
   <si>
     <t>Name</t>
   </si>
@@ -320,9 +320,6 @@
     <t>DRAKE SOLAR SOLUTIONS LLC</t>
   </si>
   <si>
-    <t>854-219-2357</t>
-  </si>
-  <si>
     <t>PRO SOLAR SOLUTIONS LLC</t>
   </si>
   <si>
@@ -507,6 +504,12 @@
   </si>
   <si>
     <t>This dealer covers all of iowa and some of west IL </t>
+  </si>
+  <si>
+    <t>Also covers all of California</t>
+  </si>
+  <si>
+    <t>843-376-9155</t>
   </si>
 </sst>
 </file>
@@ -970,7 +973,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -978,7 +981,7 @@
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>6</v>
@@ -989,7 +992,9 @@
       <c r="E2" s="2">
         <v>-95.559602999999996</v>
       </c>
-      <c r="F2" s="2"/>
+      <c r="F2" s="2" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="3" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
@@ -1135,7 +1140,7 @@
         <v>32</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D11" s="2">
         <v>28.850374804966101</v>
@@ -1169,7 +1174,7 @@
         <v>37</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D13" s="2">
         <v>21.497420327698102</v>
@@ -1203,7 +1208,7 @@
         <v>42</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D15" s="2">
         <v>33.393993764255498</v>
@@ -1336,7 +1341,7 @@
         <v>64</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>65</v>
@@ -1506,10 +1511,10 @@
         <v>94</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>95</v>
+        <v>158</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D33" s="2">
         <v>35.294231952066198</v>
@@ -1520,13 +1525,13 @@
     </row>
     <row r="34" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="C34" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>98</v>
       </c>
       <c r="D34" s="2">
         <v>39.306282000000003</v>
@@ -1537,13 +1542,13 @@
     </row>
     <row r="35" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="C35" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>101</v>
       </c>
       <c r="D35" s="2">
         <v>35.895916</v>
@@ -1554,13 +1559,13 @@
     </row>
     <row r="36" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="C36" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="D36" s="2">
         <v>38.036141000000001</v>
@@ -1571,13 +1576,13 @@
     </row>
     <row r="37" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="C37" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>107</v>
       </c>
       <c r="D37" s="2">
         <v>41.644714</v>
@@ -1588,13 +1593,13 @@
     </row>
     <row r="38" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="C38" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>110</v>
       </c>
       <c r="D38" s="2">
         <v>37.311083000000004</v>
@@ -1605,13 +1610,13 @@
     </row>
     <row r="39" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="C39" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>113</v>
       </c>
       <c r="D39" s="2">
         <v>39.789189999999998</v>
@@ -1622,13 +1627,13 @@
     </row>
     <row r="40" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="C40" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>116</v>
       </c>
       <c r="D40" s="2">
         <v>40.584440999999998</v>
@@ -1639,13 +1644,13 @@
     </row>
     <row r="41" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B41" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>118</v>
       </c>
       <c r="D41" s="2">
         <v>36.226163999999997</v>
@@ -1654,18 +1659,18 @@
         <v>-86.629830999999996</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B42" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>120</v>
       </c>
       <c r="D42" s="2">
         <v>39.748579999999997</v>
@@ -1674,18 +1679,18 @@
         <v>-105.07538</v>
       </c>
       <c r="F42" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B43" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>122</v>
       </c>
       <c r="D43" s="2">
         <v>28.81718</v>
@@ -1694,7 +1699,7 @@
         <v>-81.848889999999997</v>
       </c>
       <c r="F43" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -1702,10 +1707,10 @@
         <v>66</v>
       </c>
       <c r="B44" t="s">
+        <v>122</v>
+      </c>
+      <c r="C44" t="s">
         <v>123</v>
-      </c>
-      <c r="C44" t="s">
-        <v>124</v>
       </c>
       <c r="D44">
         <v>35.174399899999997</v>
@@ -1714,18 +1719,18 @@
         <v>-80.904181699999995</v>
       </c>
       <c r="F44" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
+        <v>124</v>
+      </c>
+      <c r="B45" t="s">
         <v>125</v>
       </c>
-      <c r="B45" t="s">
+      <c r="C45" t="s">
         <v>126</v>
-      </c>
-      <c r="C45" t="s">
-        <v>127</v>
       </c>
       <c r="D45">
         <v>33.466299999999997</v>
@@ -1736,13 +1741,13 @@
     </row>
     <row r="46" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
+        <v>127</v>
+      </c>
+      <c r="B46" t="s">
         <v>128</v>
       </c>
-      <c r="B46" t="s">
+      <c r="C46" t="s">
         <v>129</v>
-      </c>
-      <c r="C46" t="s">
-        <v>130</v>
       </c>
       <c r="D46" s="3">
         <v>34.587166000000003</v>
@@ -1753,13 +1758,13 @@
     </row>
     <row r="47" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
+        <v>130</v>
+      </c>
+      <c r="B47" t="s">
         <v>131</v>
       </c>
-      <c r="B47" t="s">
+      <c r="C47" t="s">
         <v>132</v>
-      </c>
-      <c r="C47" t="s">
-        <v>133</v>
       </c>
       <c r="D47" s="3">
         <v>38.957118000000001</v>
@@ -1770,13 +1775,13 @@
     </row>
     <row r="48" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
+        <v>141</v>
+      </c>
+      <c r="B48" t="s">
         <v>142</v>
       </c>
-      <c r="B48" t="s">
-        <v>143</v>
-      </c>
       <c r="C48" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D48">
         <v>37.304490000000001</v>
@@ -1785,18 +1790,18 @@
         <v>-80.036469999999994</v>
       </c>
       <c r="F48" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
+        <v>149</v>
+      </c>
+      <c r="B49" t="s">
         <v>150</v>
       </c>
-      <c r="B49" t="s">
-        <v>151</v>
-      </c>
       <c r="C49" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D49">
         <v>30.425978374733798</v>
@@ -1807,13 +1812,13 @@
     </row>
     <row r="50" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="B50" t="s">
         <v>154</v>
       </c>
-      <c r="B50" t="s">
+      <c r="C50" t="s">
         <v>155</v>
-      </c>
-      <c r="C50" t="s">
-        <v>156</v>
       </c>
       <c r="D50">
         <v>41.689357431787499</v>
@@ -1822,7 +1827,7 @@
         <v>-91.664268445845593</v>
       </c>
       <c r="F50" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -2776,7 +2781,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:E1 A51:E997 A24:E32 A3:E10 A2 C2:E2 B43 D43:E43 B42:E42 B41:E41 C23:E23 A12:E12 A11:B11 A14:E14 A13:B13 A16:E22 A15:B15 A34:E40 A33:B33" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:E1 A51:E997 A24:E32 A3:E10 A2 C2:E2 B43 D43:E43 B42:E42 B41:E41 C23:E23 A12:E12 A11:B11 A14:E14 A13:B13 A16:E22 A15:B15 A34:E40 A33" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added 3 dealers: Solar Ninja's, I Love My Solar, Virginia Inc. and Intelligent Design Heating & Cooling
</commit_message>
<xml_diff>
--- a/drive-time-locator/Backend/locations_with_coords.xlsx
+++ b/drive-time-locator/Backend/locations_with_coords.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olivier.d\.vscode\closest-dealer-api\drive-time-locator\Backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0519946-D867-4DF7-8B21-0C0802DFEE28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D66EB422-397D-4EE3-9A45-740F96101042}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="170">
   <si>
     <t>Name</t>
   </si>
@@ -510,6 +510,39 @@
   </si>
   <si>
     <t>843-376-9155</t>
+  </si>
+  <si>
+    <t>I Love My Solar, Virginia Inc.</t>
+  </si>
+  <si>
+    <t>2224 GRACE ST CHESAPEAKE, VA 23323-4051 US</t>
+  </si>
+  <si>
+    <t>877.607.6527</t>
+  </si>
+  <si>
+    <t>Solar Ninjas</t>
+  </si>
+  <si>
+    <t>1318 WANAKA ST HONOLULU, HI 96818-1134 US</t>
+  </si>
+  <si>
+    <t>This Dealer services all of Oahu </t>
+  </si>
+  <si>
+    <t>Intelligent Design Heating &amp; Cooling</t>
+  </si>
+  <si>
+    <t>1145 East Fort Lowell Road Tucson, AZ 85719 United States</t>
+  </si>
+  <si>
+    <t>This Dealer services the tuscon metro area</t>
+  </si>
+  <si>
+    <t>(808) 492-2236</t>
+  </si>
+  <si>
+    <t>(585) 309-9065</t>
   </si>
 </sst>
 </file>
@@ -1830,9 +1863,57 @@
         <v>156</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="52" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="53" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="51" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>159</v>
+      </c>
+      <c r="B51" t="s">
+        <v>161</v>
+      </c>
+      <c r="C51" t="s">
+        <v>160</v>
+      </c>
+      <c r="D51">
+        <v>36.746559898694997</v>
+      </c>
+      <c r="E51">
+        <v>-76.328567609906997</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>162</v>
+      </c>
+      <c r="B52" t="s">
+        <v>168</v>
+      </c>
+      <c r="C52" t="s">
+        <v>163</v>
+      </c>
+      <c r="D52">
+        <v>21.354969832653602</v>
+      </c>
+      <c r="E52">
+        <v>-157.922082919665</v>
+      </c>
+      <c r="F52" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>165</v>
+      </c>
+      <c r="B53" t="s">
+        <v>169</v>
+      </c>
+      <c r="C53" t="s">
+        <v>166</v>
+      </c>
+      <c r="F53" t="s">
+        <v>167</v>
+      </c>
+    </row>
     <row r="54" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="55" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="56" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -2781,7 +2862,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:E1 A51:E997 A24:E32 A3:E10 A2 C2:E2 B43 D43:E43 B42:E42 B41:E41 C23:E23 A12:E12 A11:B11 A14:E14 A13:B13 A16:E22 A15:B15 A34:E40 A33" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:E1 A54:E997 A24:E32 A3:E10 A2 C2:E2 B43 D43:E43 B42:E42 B41:E41 C23:E23 A12:E12 A11:B11 A14:E14 A13:B13 A16:E22 A15:B15 A34:E40 A33 D53:E53" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added 1 dealer Kyles Ultimate Energy
</commit_message>
<xml_diff>
--- a/drive-time-locator/Backend/locations_with_coords.xlsx
+++ b/drive-time-locator/Backend/locations_with_coords.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olivier.d\.vscode\closest-dealer-api\drive-time-locator\Backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7583B0F8-6732-41FE-891F-29FDD9862893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E764E45-04EF-4235-BFBD-A09E2C285E32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="19290" windowHeight="11230" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="760" yWindow="760" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="173">
   <si>
     <t>Name</t>
   </si>
@@ -543,6 +543,15 @@
   </si>
   <si>
     <t>(585) 309-9065</t>
+  </si>
+  <si>
+    <t>Kyles Ultimate Energy</t>
+  </si>
+  <si>
+    <t>(469) 451-0042</t>
+  </si>
+  <si>
+    <t>6004 Meadowside Trail, Arlington, TX 76017, USA</t>
   </si>
 </sst>
 </file>
@@ -1920,7 +1929,23 @@
         <v>167</v>
       </c>
     </row>
-    <row r="54" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="54" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>170</v>
+      </c>
+      <c r="B54" t="s">
+        <v>171</v>
+      </c>
+      <c r="C54" t="s">
+        <v>172</v>
+      </c>
+      <c r="D54">
+        <v>32.647732573717803</v>
+      </c>
+      <c r="E54">
+        <v>-97.120585303843399</v>
+      </c>
+    </row>
     <row r="55" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="56" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="57" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -2868,7 +2893,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:E1 A54:E997 A24:E32 A3:E10 A2 C2:E2 B43 D43:E43 B42:E42 B41:E41 C23:E23 A12:E12 A11:B11 A14:E14 A13:B13 A16:E22 A15:B15 A34:E40 A33" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:E1 A55:E997 A24:E32 A3:E10 A2 C2:E2 B43 D43:E43 B42:E42 B41:E41 C23:E23 A12:E12 A11:B11 A14:E14 A13:B13 A16:E22 A15:B15 A34:E40 A33" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added 1 more dealer Cardinal Power Systems L.L.C.
</commit_message>
<xml_diff>
--- a/drive-time-locator/Backend/locations_with_coords.xlsx
+++ b/drive-time-locator/Backend/locations_with_coords.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olivier.d\.vscode\closest-dealer-api\drive-time-locator\Backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E764E45-04EF-4235-BFBD-A09E2C285E32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF646A30-3956-4F0C-A943-B40FA4C77F8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="176">
   <si>
     <t>Name</t>
   </si>
@@ -59,171 +59,111 @@
     <t>JUAPI PROJECT SERVICES, LLC</t>
   </si>
   <si>
-    <t>7875906560</t>
-  </si>
-  <si>
     <t>#3 CALLE ACACIA OFICINA 201-B, SAN JUAN, PR, 920</t>
   </si>
   <si>
     <t>JACKSON ELECTRIC, LLC</t>
   </si>
   <si>
-    <t>8088754464</t>
-  </si>
-  <si>
     <t>171 AUHANA RD, KIHEI, HI, 96753</t>
   </si>
   <si>
     <t>HI-POWER SOLAR</t>
   </si>
   <si>
-    <t>8088880027</t>
-  </si>
-  <si>
     <t>98-723 KUAHAO PL STE A13, PEARL CITY, HI, 96782</t>
   </si>
   <si>
     <t>BLUESKY ENERGY LLC</t>
   </si>
   <si>
-    <t>8088955816</t>
-  </si>
-  <si>
     <t>16-711 MILO ST UNIT B, KEAAU, HI, 96749</t>
   </si>
   <si>
     <t>KINGDOM SOLAR INC</t>
   </si>
   <si>
-    <t>9254818903</t>
-  </si>
-  <si>
     <t>3989 1ST ST STE E, LIVERMORE, CA, 94551</t>
   </si>
   <si>
     <t>Sun Driven Solar LLC</t>
   </si>
   <si>
-    <t>2088100541 Cesar 208-994-9870</t>
-  </si>
-  <si>
     <t>10604 N PALISADES WAY, BOISE, ID, 83714</t>
   </si>
   <si>
     <t>ROCKNOLL ENERGY SYSTEMS, INC</t>
   </si>
   <si>
-    <t>5133798974</t>
-  </si>
-  <si>
     <t>6344 US RT 22-3, MORROW, OH, 45152</t>
   </si>
   <si>
     <t>SOLERA ENERGY LLC</t>
   </si>
   <si>
-    <t>4177715817</t>
-  </si>
-  <si>
     <t>1725 N PACKER RD, SPRINGFIELD, MO, 65803</t>
   </si>
   <si>
     <t>KR.SOLAR LLC DBA LOTUS SOLAR &amp; ENERGY</t>
   </si>
   <si>
-    <t>4073777437</t>
-  </si>
-  <si>
     <t>All Circuit Electrical L.L.C.</t>
   </si>
   <si>
-    <t>2609978336</t>
-  </si>
-  <si>
     <t>5510 N. HWY 27, BRYANT, IN, 47326-8835</t>
   </si>
   <si>
     <t>7 Star Electric</t>
   </si>
   <si>
-    <t>8083068919</t>
-  </si>
-  <si>
     <t>MICHIGAN SOLAR SOLUTIONS INC</t>
   </si>
   <si>
-    <t>2489233456</t>
-  </si>
-  <si>
     <t>3260 OLD FARM LN, COMMERCE, MI, 48390</t>
   </si>
   <si>
     <t>VECTOR ENERGY LLC DBA FUSION POWER</t>
   </si>
   <si>
-    <t>6023696969</t>
-  </si>
-  <si>
     <t>Riverside Electric</t>
   </si>
   <si>
-    <t>+1 513-936-0100</t>
-  </si>
-  <si>
     <t>680 Redna Terrace, Cincinnati, OH, 45215</t>
   </si>
   <si>
     <t>PV HAWAII LLC</t>
   </si>
   <si>
-    <t>8087977210</t>
-  </si>
-  <si>
     <t>91-6221 KAPOLEI PARKWAY UNIT 11, EWA BEACH, HI, 96706</t>
   </si>
   <si>
     <t>OREGON SOLAR CLEAN LLC</t>
   </si>
   <si>
-    <t>5415254250</t>
-  </si>
-  <si>
     <t>35 OWOSSO DR, EUGENE, OR, 97404-2628</t>
   </si>
   <si>
     <t>TOPVIEW SOLAR INC</t>
   </si>
   <si>
-    <t>7147279535</t>
-  </si>
-  <si>
     <t>14500 ROSCOE BLVD 4TH FLOOR, PANORAMA CITY, CA, 91402</t>
   </si>
   <si>
     <t>JACKSON SOLAR LLC</t>
   </si>
   <si>
-    <t>573-243-7657</t>
-  </si>
-  <si>
     <t>127 W MAIN ST APT A, JACKSON, MO, 63755-1879</t>
   </si>
   <si>
     <t>HUNTINPARTY LLC DBA CARBON RECALL INDEPENDENCE</t>
   </si>
   <si>
-    <t>3195217591</t>
-  </si>
-  <si>
     <t>132 TERRACE DR, INDEPENDENCE, IA, 50644</t>
   </si>
   <si>
     <t>United Better Homes, LLC</t>
   </si>
   <si>
-    <t>4012740111</t>
-  </si>
-  <si>
     <t>535 PINE ST, CENTRAL FALLS, RI, 2863</t>
   </si>
   <si>
@@ -239,81 +179,54 @@
     <t>CLEAN ENERGY INNOVATORS LLC</t>
   </si>
   <si>
-    <t>206-965-8666</t>
-  </si>
-  <si>
     <t>12914 SE 257TH ST, KENT, WA, 98030</t>
   </si>
   <si>
     <t>HARDWARE RIVER COMPANY LLC</t>
   </si>
   <si>
-    <t>4348721564</t>
-  </si>
-  <si>
     <t>4363 BURTON LN, NORTH GARDEN, VA, 22959</t>
   </si>
   <si>
     <t>POWER PRO LLC</t>
   </si>
   <si>
-    <t>4196022408</t>
-  </si>
-  <si>
     <t>10415 HARMON RD, BERLIN HEIGHTS, OH, 44814</t>
   </si>
   <si>
     <t>VISIONS DESIGN ELECTRICAL &amp; CONSTRUCTION LLC</t>
   </si>
   <si>
-    <t>4696938668</t>
-  </si>
-  <si>
     <t>841 WATSON LN W, NEW BRAUNFELS, TX, 78130</t>
   </si>
   <si>
     <t>HOOSIER SOLAR SOLUTIONS LLC</t>
   </si>
   <si>
-    <t>8123207056</t>
-  </si>
-  <si>
     <t>903 S DEER RUN, ELLETTSVILLE, IN, 47429</t>
   </si>
   <si>
     <t>JUDD SOLAR LLC DBA BONE DRY SOLAR</t>
   </si>
   <si>
-    <t>3177428460</t>
-  </si>
-  <si>
     <t>7735 WINTON DR, INDIANAPOLIS, IN, 46268</t>
   </si>
   <si>
     <t>HOME RENEWABLES LLC DBA AKINO SOLAR</t>
   </si>
   <si>
-    <t>8653511080</t>
-  </si>
-  <si>
     <t>9285 UPSTREAM LN, KNOXVILLE, TN, 37931</t>
   </si>
   <si>
     <t>ATLAS GENERAL CONSTRUCTION INC DBA ATLAS CLEAN ENERGY</t>
   </si>
   <si>
-    <t>9168796187</t>
-  </si>
-  <si>
     <t>930 BONNIE LN, AUBURN, CA, 95603-9452</t>
   </si>
   <si>
     <t>QTS SOLAR LLC</t>
   </si>
   <si>
-    <t>3309888063</t>
-  </si>
-  <si>
     <t>138 STERLING AVE, RITTMAN, OH, 44270-1655</t>
   </si>
   <si>
@@ -323,45 +236,30 @@
     <t>PRO SOLAR SOLUTIONS LLC</t>
   </si>
   <si>
-    <t>7203383818</t>
-  </si>
-  <si>
     <t>9756 TALL TIMBER DR, WEST CHESTER, OH, 45241-1221</t>
   </si>
   <si>
     <t>SOUTHERN ENERGY MANAGEMENT INC</t>
   </si>
   <si>
-    <t>9196040224</t>
-  </si>
-  <si>
     <t>5908 TRIANGLE DR, RALEIGH, NC, 27617</t>
   </si>
   <si>
     <t>TIGER SOLAR COMPANY</t>
   </si>
   <si>
-    <t>4342933763</t>
-  </si>
-  <si>
     <t>1132 E MARKET ST BAY 5, CHARLOTTESVILLE, VA, 22902-5351</t>
   </si>
   <si>
     <t>INDEPENDENCE RENEWABLE ENERGY LLC</t>
   </si>
   <si>
-    <t>8154141788</t>
-  </si>
-  <si>
     <t>926 E CHURCH ST, SANDWICH, IL, 60548</t>
   </si>
   <si>
     <t>Suntalk Solar</t>
   </si>
   <si>
-    <t xml:space="preserve">(303) 904-2268 </t>
-  </si>
-  <si>
     <t>27846 US-550, Durango, CO 81301, USA</t>
   </si>
   <si>
@@ -467,9 +365,6 @@
     <t>Willing to travel 300 miles from Salem </t>
   </si>
   <si>
-    <t>865-314-7040</t>
-  </si>
-  <si>
     <t>19400 Florida 44 Eustis, FL 32736 United States</t>
   </si>
   <si>
@@ -509,18 +404,12 @@
     <t>Also covers all of California</t>
   </si>
   <si>
-    <t>843-376-9155</t>
-  </si>
-  <si>
     <t>I Love My Solar, Virginia Inc.</t>
   </si>
   <si>
     <t>2224 GRACE ST CHESAPEAKE, VA 23323-4051 US</t>
   </si>
   <si>
-    <t>877.607.6527</t>
-  </si>
-  <si>
     <t>Solar Ninjas</t>
   </si>
   <si>
@@ -552,16 +441,137 @@
   </si>
   <si>
     <t>6004 Meadowside Trail, Arlington, TX 76017, USA</t>
+  </si>
+  <si>
+    <t>Cardinal Power Systems L.L.C.</t>
+  </si>
+  <si>
+    <t>3706 Gleneden Dr, Lansing, MI 48906, USA</t>
+  </si>
+  <si>
+    <t>(517) 490-1240</t>
+  </si>
+  <si>
+    <t>(787) 590-6560</t>
+  </si>
+  <si>
+    <t>(808) 875-4464</t>
+  </si>
+  <si>
+    <t>(808) 888-0027</t>
+  </si>
+  <si>
+    <t>(808) 895-5816</t>
+  </si>
+  <si>
+    <t>(925) 481-8903</t>
+  </si>
+  <si>
+    <t>(208) 810-0541, Cesar (208) 994-9870</t>
+  </si>
+  <si>
+    <t>(513) 379-8974</t>
+  </si>
+  <si>
+    <t>(417) 771-5817</t>
+  </si>
+  <si>
+    <t>(407) 377-7437</t>
+  </si>
+  <si>
+    <t>(260) 997-8336</t>
+  </si>
+  <si>
+    <t>(808) 306-8919</t>
+  </si>
+  <si>
+    <t>(248) 923-3456</t>
+  </si>
+  <si>
+    <t>(602) 369-6969</t>
+  </si>
+  <si>
+    <t>(513) 936-0100</t>
+  </si>
+  <si>
+    <t>(808) 797-7210</t>
+  </si>
+  <si>
+    <t>(541) 525-4250</t>
+  </si>
+  <si>
+    <t>(714) 727-9535</t>
+  </si>
+  <si>
+    <t>(573) 243-7657</t>
+  </si>
+  <si>
+    <t>(319) 521-7591</t>
+  </si>
+  <si>
+    <t>(401) 274-0111</t>
+  </si>
+  <si>
+    <t>(865) 314-7040</t>
+  </si>
+  <si>
+    <t>(206) 965-8666</t>
+  </si>
+  <si>
+    <t>(434) 872-1564</t>
+  </si>
+  <si>
+    <t>(419) 602-2408</t>
+  </si>
+  <si>
+    <t>(469) 693-8668</t>
+  </si>
+  <si>
+    <t>(812) 320-7056</t>
+  </si>
+  <si>
+    <t>(317) 742-8460</t>
+  </si>
+  <si>
+    <t>(865) 351-1080</t>
+  </si>
+  <si>
+    <t>(916) 879-6187</t>
+  </si>
+  <si>
+    <t>(330) 988-8063</t>
+  </si>
+  <si>
+    <t>(843) 376-9155</t>
+  </si>
+  <si>
+    <t>(720) 338-3818</t>
+  </si>
+  <si>
+    <t>(919) 604-0224</t>
+  </si>
+  <si>
+    <t>(434) 293-3763</t>
+  </si>
+  <si>
+    <t>(815) 414-1788</t>
+  </si>
+  <si>
+    <t>(303) 904-2268</t>
+  </si>
+  <si>
+    <t>(877) 607-6527</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.00000"/>
+    <numFmt numFmtId="169" formatCode="[&lt;=9999999]###\-####;\(###\)\ ###\-####"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -587,6 +597,20 @@
       <color rgb="FF03234D"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -635,7 +659,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -646,6 +670,12 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="169" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
@@ -992,7 +1022,7 @@
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
-    <col min="2" max="2" width="12.25" customWidth="1"/>
+    <col min="2" max="2" width="12.25" style="7" customWidth="1"/>
     <col min="3" max="3" width="11.75" customWidth="1"/>
     <col min="4" max="4" width="11.08203125" customWidth="1"/>
     <col min="5" max="5" width="15.25" customWidth="1"/>
@@ -1002,7 +1032,7 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -1015,15 +1045,15 @@
         <v>4</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>133</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>151</v>
+      <c r="B2" s="8" t="s">
+        <v>116</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>6</v>
@@ -1035,18 +1065,18 @@
         <v>-95.559602999999996</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>157</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>9</v>
       </c>
       <c r="D3" s="2">
         <v>18.466329999999999</v>
@@ -1057,13 +1087,13 @@
     </row>
     <row r="4" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>12</v>
       </c>
       <c r="D4" s="2">
         <v>20.729227999999999</v>
@@ -1074,13 +1104,13 @@
     </row>
     <row r="5" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>141</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D5" s="2">
         <v>21.392209999999999</v>
@@ -1091,13 +1121,13 @@
     </row>
     <row r="6" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>17</v>
+        <v>13</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D6" s="2">
         <v>19.627331999999999</v>
@@ -1108,13 +1138,13 @@
     </row>
     <row r="7" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>20</v>
+        <v>15</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>143</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D7" s="2">
         <v>37.678100000000001</v>
@@ -1125,13 +1155,13 @@
     </row>
     <row r="8" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>23</v>
+        <v>17</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>144</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D8" s="2">
         <v>43.701984000000003</v>
@@ -1142,13 +1172,13 @@
     </row>
     <row r="9" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>26</v>
+        <v>19</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>145</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D9" s="2">
         <v>40.509236999999999</v>
@@ -1159,13 +1189,13 @@
     </row>
     <row r="10" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>29</v>
+        <v>21</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>146</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="D10" s="2">
         <v>37.227837999999998</v>
@@ -1176,13 +1206,13 @@
     </row>
     <row r="11" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>32</v>
+        <v>23</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>147</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>145</v>
+        <v>110</v>
       </c>
       <c r="D11" s="2">
         <v>28.850374804966101</v>
@@ -1193,13 +1223,13 @@
     </row>
     <row r="12" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>34</v>
+        <v>24</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>148</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D12" s="2">
         <v>35.74174</v>
@@ -1210,13 +1240,13 @@
     </row>
     <row r="13" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>37</v>
+        <v>26</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>149</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>146</v>
+        <v>111</v>
       </c>
       <c r="D13" s="2">
         <v>21.497420327698102</v>
@@ -1227,13 +1257,13 @@
     </row>
     <row r="14" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>39</v>
+        <v>27</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>150</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="D14" s="2">
         <v>42.569713</v>
@@ -1244,13 +1274,13 @@
     </row>
     <row r="15" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>42</v>
+        <v>29</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>151</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>147</v>
+        <v>112</v>
       </c>
       <c r="D15" s="2">
         <v>33.393993764255498</v>
@@ -1261,13 +1291,13 @@
     </row>
     <row r="16" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>44</v>
+        <v>30</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>152</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="D16" s="2">
         <v>39.262909000000001</v>
@@ -1278,13 +1308,13 @@
     </row>
     <row r="17" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>47</v>
+        <v>32</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>153</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="D17" s="2">
         <v>21.325071999999999</v>
@@ -1295,13 +1325,13 @@
     </row>
     <row r="18" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>50</v>
+        <v>34</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>154</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="D18" s="2">
         <v>44.092323</v>
@@ -1312,13 +1342,13 @@
     </row>
     <row r="19" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>53</v>
+        <v>36</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>155</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="D19" s="2">
         <v>34.221238</v>
@@ -1329,13 +1359,13 @@
     </row>
     <row r="20" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>56</v>
+        <v>38</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>156</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="D20" s="2">
         <v>37.383606999999998</v>
@@ -1346,13 +1376,13 @@
     </row>
     <row r="21" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>59</v>
+        <v>40</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>157</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D21" s="2">
         <v>42.467131999999999</v>
@@ -1363,13 +1393,13 @@
     </row>
     <row r="22" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>62</v>
+        <v>42</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>158</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>63</v>
+        <v>43</v>
       </c>
       <c r="D22" s="2">
         <v>41.884461999999999</v>
@@ -1380,13 +1410,13 @@
     </row>
     <row r="23" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>144</v>
+        <v>44</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>159</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="D23" s="2">
         <v>36.153689999999997</v>
@@ -1397,13 +1427,13 @@
     </row>
     <row r="24" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>68</v>
+        <v>47</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>160</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>69</v>
+        <v>48</v>
       </c>
       <c r="D24" s="2">
         <v>47.371457999999997</v>
@@ -1414,13 +1444,13 @@
     </row>
     <row r="25" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>71</v>
+        <v>49</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>161</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>72</v>
+        <v>50</v>
       </c>
       <c r="D25" s="2">
         <v>37.9407</v>
@@ -1431,13 +1461,13 @@
     </row>
     <row r="26" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>74</v>
+        <v>51</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>162</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="D26" s="2">
         <v>41.323565000000002</v>
@@ -1448,13 +1478,13 @@
     </row>
     <row r="27" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>77</v>
+        <v>53</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>163</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>78</v>
+        <v>54</v>
       </c>
       <c r="D27" s="2">
         <v>29.694703000000001</v>
@@ -1465,13 +1495,13 @@
     </row>
     <row r="28" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>80</v>
+        <v>55</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>164</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>81</v>
+        <v>56</v>
       </c>
       <c r="D28" s="2">
         <v>39.219279999999998</v>
@@ -1482,13 +1512,13 @@
     </row>
     <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>83</v>
+        <v>57</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>165</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>84</v>
+        <v>58</v>
       </c>
       <c r="D29" s="2">
         <v>39.89385</v>
@@ -1499,13 +1529,13 @@
     </row>
     <row r="30" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>86</v>
+        <v>59</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>166</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>87</v>
+        <v>60</v>
       </c>
       <c r="D30" s="2">
         <v>35.973011</v>
@@ -1516,13 +1546,13 @@
     </row>
     <row r="31" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>89</v>
+        <v>61</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>167</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>90</v>
+        <v>62</v>
       </c>
       <c r="D31" s="2">
         <v>38.898076000000003</v>
@@ -1533,13 +1563,13 @@
     </row>
     <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>92</v>
+        <v>63</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>168</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>93</v>
+        <v>64</v>
       </c>
       <c r="D32" s="2">
         <v>40.966545000000004</v>
@@ -1550,13 +1580,13 @@
     </row>
     <row r="33" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>158</v>
+        <v>65</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>169</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>148</v>
+        <v>113</v>
       </c>
       <c r="D33" s="2">
         <v>35.294231952066198</v>
@@ -1567,13 +1597,13 @@
     </row>
     <row r="34" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>96</v>
+        <v>66</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>170</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>97</v>
+        <v>67</v>
       </c>
       <c r="D34" s="2">
         <v>39.306282000000003</v>
@@ -1584,13 +1614,13 @@
     </row>
     <row r="35" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>99</v>
+        <v>68</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>171</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>100</v>
+        <v>69</v>
       </c>
       <c r="D35" s="2">
         <v>35.895916</v>
@@ -1601,13 +1631,13 @@
     </row>
     <row r="36" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>102</v>
+        <v>70</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>172</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>103</v>
+        <v>71</v>
       </c>
       <c r="D36" s="2">
         <v>38.036141000000001</v>
@@ -1618,13 +1648,13 @@
     </row>
     <row r="37" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>105</v>
+        <v>72</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>173</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>106</v>
+        <v>73</v>
       </c>
       <c r="D37" s="2">
         <v>41.644714</v>
@@ -1635,13 +1665,13 @@
     </row>
     <row r="38" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>108</v>
+        <v>74</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>174</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>109</v>
+        <v>75</v>
       </c>
       <c r="D38" s="2">
         <v>37.311083000000004</v>
@@ -1652,13 +1682,13 @@
     </row>
     <row r="39" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>111</v>
+        <v>76</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>77</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>112</v>
+        <v>78</v>
       </c>
       <c r="D39" s="2">
         <v>39.789189999999998</v>
@@ -1669,13 +1699,13 @@
     </row>
     <row r="40" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>114</v>
+        <v>79</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>80</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
       <c r="D40" s="2">
         <v>40.584440999999998</v>
@@ -1686,13 +1716,13 @@
     </row>
     <row r="41" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>116</v>
+        <v>105</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>82</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>117</v>
+        <v>83</v>
       </c>
       <c r="D41" s="2">
         <v>36.226163999999997</v>
@@ -1701,18 +1731,18 @@
         <v>-86.629830999999996</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>134</v>
+        <v>100</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>118</v>
+        <v>104</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>84</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>119</v>
+        <v>85</v>
       </c>
       <c r="D42" s="2">
         <v>39.748579999999997</v>
@@ -1721,18 +1751,18 @@
         <v>-105.07538</v>
       </c>
       <c r="F42" t="s">
-        <v>134</v>
+        <v>100</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>120</v>
+        <v>103</v>
+      </c>
+      <c r="B43" s="8" t="s">
+        <v>86</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>121</v>
+        <v>87</v>
       </c>
       <c r="D43" s="2">
         <v>28.81718</v>
@@ -1741,18 +1771,18 @@
         <v>-81.848889999999997</v>
       </c>
       <c r="F43" t="s">
-        <v>135</v>
+        <v>101</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>66</v>
-      </c>
-      <c r="B44" t="s">
-        <v>122</v>
+        <v>46</v>
+      </c>
+      <c r="B44" s="9" t="s">
+        <v>88</v>
       </c>
       <c r="C44" t="s">
-        <v>123</v>
+        <v>89</v>
       </c>
       <c r="D44">
         <v>35.174399899999997</v>
@@ -1761,18 +1791,18 @@
         <v>-80.904181699999995</v>
       </c>
       <c r="F44" t="s">
-        <v>136</v>
+        <v>102</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>124</v>
-      </c>
-      <c r="B45" t="s">
-        <v>125</v>
+        <v>90</v>
+      </c>
+      <c r="B45" s="9" t="s">
+        <v>91</v>
       </c>
       <c r="C45" t="s">
-        <v>126</v>
+        <v>92</v>
       </c>
       <c r="D45">
         <v>33.466299999999997</v>
@@ -1783,13 +1813,13 @@
     </row>
     <row r="46" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>127</v>
-      </c>
-      <c r="B46" t="s">
-        <v>128</v>
+        <v>93</v>
+      </c>
+      <c r="B46" s="9" t="s">
+        <v>94</v>
       </c>
       <c r="C46" t="s">
-        <v>129</v>
+        <v>95</v>
       </c>
       <c r="D46" s="3">
         <v>34.587166000000003</v>
@@ -1800,13 +1830,13 @@
     </row>
     <row r="47" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>130</v>
-      </c>
-      <c r="B47" t="s">
-        <v>131</v>
+        <v>96</v>
+      </c>
+      <c r="B47" s="9" t="s">
+        <v>97</v>
       </c>
       <c r="C47" t="s">
-        <v>132</v>
+        <v>98</v>
       </c>
       <c r="D47" s="3">
         <v>38.957118000000001</v>
@@ -1817,13 +1847,13 @@
     </row>
     <row r="48" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>141</v>
-      </c>
-      <c r="B48" t="s">
-        <v>142</v>
+        <v>107</v>
+      </c>
+      <c r="B48" s="9" t="s">
+        <v>108</v>
       </c>
       <c r="C48" t="s">
-        <v>140</v>
+        <v>106</v>
       </c>
       <c r="D48">
         <v>37.304490000000001</v>
@@ -1832,18 +1862,18 @@
         <v>-80.036469999999994</v>
       </c>
       <c r="F48" t="s">
-        <v>143</v>
+        <v>109</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>149</v>
-      </c>
-      <c r="B49" t="s">
-        <v>150</v>
+        <v>114</v>
+      </c>
+      <c r="B49" s="9" t="s">
+        <v>115</v>
       </c>
       <c r="C49" t="s">
-        <v>152</v>
+        <v>117</v>
       </c>
       <c r="D49">
         <v>30.425978374733798</v>
@@ -1854,13 +1884,13 @@
     </row>
     <row r="50" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="B50" t="s">
-        <v>154</v>
+        <v>118</v>
+      </c>
+      <c r="B50" s="9" t="s">
+        <v>119</v>
       </c>
       <c r="C50" t="s">
-        <v>155</v>
+        <v>120</v>
       </c>
       <c r="D50">
         <v>41.689357431787499</v>
@@ -1869,18 +1899,18 @@
         <v>-91.664268445845593</v>
       </c>
       <c r="F50" t="s">
-        <v>156</v>
+        <v>121</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>159</v>
-      </c>
-      <c r="B51" t="s">
-        <v>161</v>
+        <v>123</v>
+      </c>
+      <c r="B51" s="9" t="s">
+        <v>175</v>
       </c>
       <c r="C51" t="s">
-        <v>160</v>
+        <v>124</v>
       </c>
       <c r="D51">
         <v>36.746559898694997</v>
@@ -1891,13 +1921,13 @@
     </row>
     <row r="52" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>162</v>
-      </c>
-      <c r="B52" t="s">
-        <v>168</v>
+        <v>125</v>
+      </c>
+      <c r="B52" s="9" t="s">
+        <v>131</v>
       </c>
       <c r="C52" t="s">
-        <v>163</v>
+        <v>126</v>
       </c>
       <c r="D52">
         <v>21.354969832653602</v>
@@ -1906,18 +1936,18 @@
         <v>-157.922082919665</v>
       </c>
       <c r="F52" t="s">
-        <v>164</v>
+        <v>127</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>165</v>
-      </c>
-      <c r="B53" t="s">
-        <v>169</v>
+        <v>128</v>
+      </c>
+      <c r="B53" s="9" t="s">
+        <v>132</v>
       </c>
       <c r="C53" t="s">
-        <v>166</v>
+        <v>129</v>
       </c>
       <c r="D53">
         <v>32.2655031017566</v>
@@ -1926,18 +1956,18 @@
         <v>-110.954090261619</v>
       </c>
       <c r="F53" t="s">
-        <v>167</v>
+        <v>130</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>170</v>
-      </c>
-      <c r="B54" t="s">
-        <v>171</v>
+        <v>133</v>
+      </c>
+      <c r="B54" s="9" t="s">
+        <v>134</v>
       </c>
       <c r="C54" t="s">
-        <v>172</v>
+        <v>135</v>
       </c>
       <c r="D54">
         <v>32.647732573717803</v>
@@ -1946,7 +1976,23 @@
         <v>-97.120585303843399</v>
       </c>
     </row>
-    <row r="55" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="55" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>136</v>
+      </c>
+      <c r="B55" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="C55" t="s">
+        <v>137</v>
+      </c>
+      <c r="D55">
+        <v>42.761920501893698</v>
+      </c>
+      <c r="E55">
+        <v>-84.600225889876896</v>
+      </c>
+    </row>
     <row r="56" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="57" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="58" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -2893,7 +2939,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:E1 A55:E997 A24:E32 A3:E10 A2 C2:E2 B43 D43:E43 B42:E42 B41:E41 C23:E23 A12:E12 A11:B11 A14:E14 A13:B13 A16:E22 A15:B15 A34:E40 A33" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:E1 A56:E997 A24:A32 A3:A10 A2 C2:E2 D43:E43 C42:E42 C41:E41 C23:E23 A12 A11 A14 A13 A16:A22 A15 A34:A40 A33 C24:E32 C3:E10 C12:E12 C14:E14 C16:E22 C34:E40" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>